<commit_message>
Se agrega el caso de test de las tarjetas CON Jest
</commit_message>
<xml_diff>
--- a/docs/planificacion/lista-requerimientos.xlsx
+++ b/docs/planificacion/lista-requerimientos.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referencias" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$2:$U$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$2:$U$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U50"/>
+  <dimension ref="A1:U52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -777,7 +777,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>El usuario crea su cuenta con nombre completo, usuario, correo y contraseña (mínimo 8 caracteres, con mayúscula, minúscula y número) y puede indicar que se registra como empresa.</t>
+          <t>El usuario crea su cuenta con correo, nombre de usuario y contraseña (mínimo 6 caracteres, con mayúscula, minúscula y número, repetida para confirmar) y elige si sólo compra, vende como particular o vende como empresa.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>El comprador busca por texto y filtra por categoría (leída de la tabla categorías) y por talle.</t>
+          <t>El comprador busca por texto y filtra por categoría (leída de la tabla categorías), por talle y por público (Adulto, Femenino, Masculino, Infantil o Unisex).</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>El comprador ve fotos, precio con descuento, talles, descripción, disponibilidad y el vendedor de la prenda.</t>
+          <t>El comprador ve fotos, precio con descuento, talles, descripción, condición (nueva o usada), disponibilidad y el vendedor de la prenda.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>El usuario marca prendas con un corazón y las ve en la pestaña Favoritos.</t>
+          <t>El usuario marca prendas con una estrella y las ve en la pestaña Favoritos.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Sin HU en Etapa 1 (pendiente de agregar).</t>
+          <t>Etapa 1: HU22. Por ahora se guardan sólo mientras la app está abierta.</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="S13" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>HU22</t>
         </is>
       </c>
       <c r="T13" s="4" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>El vendedor carga título, descripción (hasta 30 caracteres), precio (35.000 o 35,50), categoría, talles por chips y hasta 5 fotos desde la cámara o la galería.</t>
+          <t>El vendedor carga título, descripción (hasta 500 caracteres), condición (nuevo o usado), uno o más públicos (Adulto, Femenino, Masculino, Infantil, Unisex), precio (35.000 o 35,50), categoría, talles por chips y hasta 5 fotos desde la cámara o la galería.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: HU06, RF3. Zod + RHF, imágenes en Supabase Storage.</t>
+          <t>Etapa 1: HU06, RF3. Zod + RHF, imágenes en Supabase Storage. Condición y público múltiple: migración 18 (27/10).</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="R15" s="6" t="inlineStr">
         <is>
-          <t>RF-039</t>
+          <t>RF-038</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
@@ -2590,41 +2590,41 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Medio de pago simulado</t>
+          <t>Medios de pago</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>El comprador elige el medio de pago; el pago es lógico, sin pasarela real (Won't W1).</t>
+          <t>El comprador elige Efectivo, Tarjeta de crédito, Tarjeta de débito o Mercado Pago. Las tarjetas se cargan en un formulario propio y las valida una API de tarjetas propia simulada (Luhn, marca, vencimiento, código, DNI y tipo de tarjeta); se guardan sólo marca, últimos 4 dígitos y cuotas. Modo prueba, sin dinero real.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Frontend / Backend / Base de Datos</t>
         </is>
       </c>
       <c r="G22" s="5" t="n">
         <v>46313</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>46313</v>
+        <v>46323</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: HU12.</t>
+          <t>Etapa 1: HU12. 28/10: se quitó la transferencia; Edge Function pago-tarjeta y migración 19.</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3/2/1</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
-          <t>1/0,5/0,5</t>
+          <t>3/2/1</t>
         </is>
       </c>
       <c r="M22" s="6" t="inlineStr">
@@ -2634,12 +2634,12 @@
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
-          <t>1/0,5/0,5</t>
+          <t>2/1/1</t>
         </is>
       </c>
       <c r="P22" s="6" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="T22" s="4" t="inlineStr">
         <is>
-          <t>TC-HU12-01; Maestro 05</t>
+          <t>TC-HU12-01; TC-PAGO-01..08; Jest tarjeta, FormularioTarjeta; Maestro 05</t>
         </is>
       </c>
       <c r="U22" s="6" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Al confirmar, el comprador recibe un correo con el código, los productos y los datos de entrega.</t>
+          <t>Al confirmar (o al aprobarse el pago con tarjeta o Mercado Pago), el comprador recibe un correo con el código, los productos, los datos de entrega y, con crédito, la comisión y las cuotas.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -2809,14 +2809,14 @@
         <v>46322</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Edge Function enviar-correo-compra con Resend.</t>
+          <t>Edge Function enviar-correo-compra por Gmail SMTP (GMAIL_USUARIO, GMAIL_CLAVE) con Resend de respaldo.</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="T24" s="4" t="inlineStr">
         <is>
-          <t>Planilla QA (manual)</t>
+          <t>Planilla QA (TC-MAIL-01, 02)</t>
         </is>
       </c>
       <c r="U24" s="6" t="inlineStr">
@@ -2888,46 +2888,46 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>RF-023</t>
+          <t>RF-040</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Historial de compras</t>
+          <t>Comisión y cuotas con tarjeta de crédito</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>El comprador ve sus compras con estado, fecha y total.</t>
+          <t>Pagar con crédito suma una comisión del 6% sobre productos + envío; se paga en 1, 3, 6 o 12 cuotas con interés total de 0, 10, 20 o 40%. El servidor calcula los importes.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Frontend / Base de Datos</t>
+          <t>Backend / Frontend / Base de Datos</t>
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>46279</v>
+        <v>46323</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>46313</v>
+        <v>46324</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Migración 02.</t>
+          <t>Etapa 1: HU12. comision_tarjeta_credito() en migración 19; INTERES_CUOTAS en utils/tarjeta.ts y su copia del servidor.</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2/1/0,5</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
         <is>
-          <t>2/1/1</t>
+          <t>2/1/0,5</t>
         </is>
       </c>
       <c r="M25" s="6" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="O25" s="6" t="inlineStr">
         <is>
-          <t>1/0,5/0,5</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="P25" s="6" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="Q25" s="6" t="inlineStr">
         <is>
-          <t>RF-021</t>
+          <t>RF-020, RF-021</t>
         </is>
       </c>
       <c r="R25" s="6" t="inlineStr">
@@ -2962,12 +2962,12 @@
       </c>
       <c r="S25" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>HU12</t>
         </is>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>Planilla QA (manual)</t>
+          <t>TC-PAGO-03..05; Jest tarjeta, pagosService</t>
         </is>
       </c>
       <c r="U25" s="6" t="inlineStr">
@@ -2984,56 +2984,56 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Ubicación</t>
+          <t>Carrito y compra</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>RF-024</t>
+          <t>RF-041</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Geolocalización y mapa</t>
+          <t>Pago con Mercado Pago</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>El GPS completa la dirección con aviso de precisión; si falla, se escribe a mano y se ve en un mapa de OpenStreetMap.</t>
+          <t>El comprador paga con Mercado Pago Checkout Pro (modo prueba) dentro de la app; el pago se verifica con la API y un webhook, y el pedido no avanza hasta que se acredita.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Frontend / Implementación</t>
+          <t>Backend / Frontend / Implementación</t>
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>46313</v>
+        <v>46323</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>46319</v>
+        <v>46323</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: HU17, Should S1. Se pasó de Google Maps a OpenStreetMap por costo.</t>
+          <t>Etapa 1: HU12, Won't W1 implementado en modo prueba. Edge Functions pago-mercadopago y mp-webhook.</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3/2/1</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>3/2/1</t>
+          <t>2/1/1</t>
         </is>
       </c>
       <c r="M26" s="6" t="inlineStr">
         <is>
-          <t>2/1/1</t>
+          <t>2/1/0,5</t>
         </is>
       </c>
       <c r="N26" s="6" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
-          <t>1/1/0,5</t>
+          <t>2/1/0,5</t>
         </is>
       </c>
       <c r="P26" s="6" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="Q26" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RF-020, RF-021</t>
         </is>
       </c>
       <c r="R26" s="6" t="inlineStr">
@@ -3063,12 +3063,12 @@
       </c>
       <c r="S26" s="4" t="inlineStr">
         <is>
-          <t>HU17</t>
+          <t>HU12</t>
         </is>
       </c>
       <c r="T26" s="4" t="inlineStr">
         <is>
-          <t>Jest VerEnMapa</t>
+          <t>TC-PAGO-09..11</t>
         </is>
       </c>
       <c r="U26" s="6" t="inlineStr">
@@ -3085,53 +3085,53 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Vendedores y pedidos</t>
+          <t>Carrito y compra</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>RF-025</t>
+          <t>RF-023</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Mis ventas y estado de pedidos</t>
+          <t>Historial de compras</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>El vendedor ve sus ventas y cambia el estado del pedido (preparando, enviado, entregado).</t>
+          <t>El comprador ve sus compras con estado, fecha y total.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Frontend / Backend / Base de Datos</t>
+          <t>Frontend / Base de Datos</t>
         </is>
       </c>
       <c r="G27" s="5" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H27" s="5" t="n">
         <v>46313</v>
       </c>
-      <c r="H27" s="5" t="n">
-        <v>46318</v>
-      </c>
       <c r="I27" s="6" t="n">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>Migraciones 10 y 11.</t>
+          <t>Etapa 1: HU23. Migración 02.</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L27" s="6" t="inlineStr">
+        <is>
           <t>2/1/1</t>
         </is>
       </c>
-      <c r="L27" s="6" t="inlineStr">
-        <is>
-          <t>2/1/1</t>
-        </is>
-      </c>
       <c r="M27" s="6" t="inlineStr">
         <is>
           <t>—</t>
@@ -3139,12 +3139,12 @@
       </c>
       <c r="N27" s="6" t="inlineStr">
         <is>
-          <t>1/1/0,5</t>
+          <t>1/0,5/0,5</t>
         </is>
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
-          <t>1/1/0,5</t>
+          <t>1/0,5/0,5</t>
         </is>
       </c>
       <c r="P27" s="6" t="inlineStr">
@@ -3164,12 +3164,12 @@
       </c>
       <c r="S27" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>HU23</t>
         </is>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>Jest pedidos</t>
+          <t>Planilla QA (manual)</t>
         </is>
       </c>
       <c r="U27" s="6" t="inlineStr">
@@ -3186,41 +3186,41 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Vendedores y pedidos</t>
+          <t>Ubicación</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>RF-026</t>
+          <t>RF-024</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Calificación de vendedores</t>
+          <t>Geolocalización y mapa</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>El comprador califica al vendedor después de recibir el pedido; quien no tiene opiniones se ve con 5 estrellas "(nuevo)".</t>
+          <t>El GPS completa la dirección con aviso de precisión; si falla, se escribe a mano y se ve en un mapa de OpenStreetMap.</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Frontend / Base de Datos</t>
+          <t>Frontend / Implementación</t>
         </is>
       </c>
       <c r="G28" s="5" t="n">
-        <v>46318</v>
+        <v>46313</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>Migración 12.</t>
+          <t>Etapa 1: HU17, Should S1. Se pasó de Google Maps a OpenStreetMap por costo.</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
@@ -3230,24 +3230,24 @@
       </c>
       <c r="L28" s="6" t="inlineStr">
         <is>
+          <t>3/2/1</t>
+        </is>
+      </c>
+      <c r="M28" s="6" t="inlineStr">
+        <is>
+          <t>2/1/1</t>
+        </is>
+      </c>
+      <c r="N28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O28" s="6" t="inlineStr">
+        <is>
           <t>1/1/0,5</t>
         </is>
       </c>
-      <c r="M28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N28" s="6" t="inlineStr">
-        <is>
-          <t>1/0,5/0,5</t>
-        </is>
-      </c>
-      <c r="O28" s="6" t="inlineStr">
-        <is>
-          <t>1/0,5/0,5</t>
-        </is>
-      </c>
       <c r="P28" s="6" t="inlineStr">
         <is>
           <t>—</t>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="Q28" s="6" t="inlineStr">
         <is>
-          <t>RF-025</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R28" s="6" t="inlineStr">
@@ -3265,12 +3265,12 @@
       </c>
       <c r="S28" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>HU17</t>
         </is>
       </c>
       <c r="T28" s="4" t="inlineStr">
         <is>
-          <t>Planilla QA (manual)</t>
+          <t>Jest VerEnMapa; Postman OpenStreetMap (postman/, 4 casos de Nominatim)</t>
         </is>
       </c>
       <c r="U28" s="6" t="inlineStr">
@@ -3292,61 +3292,61 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>RF-027</t>
+          <t>RF-025</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Página pública del vendedor</t>
+          <t>Mis ventas y estado de pedidos</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Cualquier usuario ve las prendas y la calificación de un vendedor sin ver sus datos personales.</t>
+          <t>El vendedor ve sus ventas y cambia el estado del pedido (preparando, enviado, entregado).</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Frontend / Base de Datos</t>
+          <t>Frontend / Backend / Base de Datos</t>
         </is>
       </c>
       <c r="G29" s="5" t="n">
+        <v>46313</v>
+      </c>
+      <c r="H29" s="5" t="n">
         <v>46318</v>
       </c>
-      <c r="H29" s="5" t="n">
-        <v>46322</v>
-      </c>
       <c r="I29" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>RNF4. Vista vendedores_publicos (migración 15).</t>
+          <t>Etapa 1: HU24. Migraciones 10 y 11.</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2/1/1</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr">
         <is>
+          <t>2/1/1</t>
+        </is>
+      </c>
+      <c r="M29" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N29" s="6" t="inlineStr">
+        <is>
           <t>1/1/0,5</t>
         </is>
       </c>
-      <c r="M29" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N29" s="6" t="inlineStr">
-        <is>
-          <t>1/0,5/0,5</t>
-        </is>
-      </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
-          <t>1/0,5/0,5</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="P29" s="6" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="Q29" s="6" t="inlineStr">
         <is>
-          <t>RF-026</t>
+          <t>RF-021</t>
         </is>
       </c>
       <c r="R29" s="6" t="inlineStr">
@@ -3366,12 +3366,12 @@
       </c>
       <c r="S29" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>HU24</t>
         </is>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>Planilla QA (manual)</t>
+          <t>Jest pedidos</t>
         </is>
       </c>
       <c r="U29" s="6" t="inlineStr">
@@ -3393,61 +3393,61 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>RF-028</t>
+          <t>RF-026</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Notificaciones push</t>
+          <t>Calificación de vendedores</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>El vendedor recibe una notificación por cada venta y el comprador por cada cambio de estado.</t>
+          <t>El comprador califica al vendedor después de recibir el pedido; quien no tiene opiniones se ve con 5 estrellas "(nuevo)".</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Backend / Implementación</t>
+          <t>Frontend / Base de Datos</t>
         </is>
       </c>
       <c r="G30" s="5" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="I30" s="6" t="n">
         <v>1</v>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>Migración 14 (pg_net). Sólo en build de EAS, no en Expo Go.</t>
+          <t>Etapa 1: HU25. Migración 12.</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>2/1/1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="M30" s="6" t="inlineStr">
         <is>
-          <t>2/1/1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N30" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1/0,5/0,5</t>
         </is>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
-          <t>2/1/0,5</t>
+          <t>1/0,5/0,5</t>
         </is>
       </c>
       <c r="P30" s="6" t="inlineStr">
@@ -3467,12 +3467,12 @@
       </c>
       <c r="S30" s="4" t="inlineStr">
         <is>
-          <t>HU19</t>
+          <t>HU25</t>
         </is>
       </c>
       <c r="T30" s="4" t="inlineStr">
         <is>
-          <t>TC-PUSH-01..05; Jest notificaciones</t>
+          <t>Planilla QA (manual)</t>
         </is>
       </c>
       <c r="U30" s="6" t="inlineStr">
@@ -3489,53 +3489,53 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Modo empresa</t>
+          <t>Vendedores y pedidos</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>RF-029</t>
+          <t>RF-027</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Alta de empresa</t>
+          <t>Página pública del vendedor</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Un usuario crea su empresa con nombre, CUIT y un enlace propio de tienda.</t>
+          <t>Cualquier usuario ve las prendas y la calificación de un vendedor sin ver sus datos personales.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Frontend / Backend / Base de Datos</t>
+          <t>Frontend / Base de Datos</t>
         </is>
       </c>
       <c r="G31" s="5" t="n">
         <v>46318</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>46318</v>
+        <v>46322</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: HU21. Migración 06.</t>
+          <t>Etapa 1: HU26, RNF4. Vista vendedores_publicos (migración 15).</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L31" s="6" t="inlineStr">
+        <is>
           <t>1/1/0,5</t>
         </is>
       </c>
-      <c r="L31" s="6" t="inlineStr">
-        <is>
-          <t>1/1/0,5</t>
-        </is>
-      </c>
       <c r="M31" s="6" t="inlineStr">
         <is>
           <t>—</t>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="N31" s="6" t="inlineStr">
         <is>
-          <t>2/1/1</t>
+          <t>1/0,5/0,5</t>
         </is>
       </c>
       <c r="O31" s="6" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="Q31" s="6" t="inlineStr">
         <is>
-          <t>RF-002</t>
+          <t>RF-026</t>
         </is>
       </c>
       <c r="R31" s="6" t="inlineStr">
@@ -3568,12 +3568,12 @@
       </c>
       <c r="S31" s="4" t="inlineStr">
         <is>
-          <t>HU21</t>
+          <t>HU26</t>
         </is>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>Jest empresas</t>
+          <t>Planilla QA (manual)</t>
         </is>
       </c>
       <c r="U31" s="6" t="inlineStr">
@@ -3590,66 +3590,66 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Modo empresa</t>
+          <t>Vendedores y pedidos</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>RF-030</t>
+          <t>RF-028</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Modo Yo / Empresa</t>
+          <t>Notificaciones push</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Un empleado elige si vende como particular o como la empresa; el propietario vende sólo como empresa; al invitarlo, el empleado queda en modo empresa.</t>
+          <t>El vendedor recibe una notificación por cada venta y el comprador por cada cambio de estado.</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Frontend / Base de Datos</t>
+          <t>Backend / Implementación</t>
         </is>
       </c>
       <c r="G32" s="5" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>46322</v>
+        <v>46319</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: HU21. Migraciones 15 y 16.</t>
+          <t>Migración 14 (pg_net). Sólo en build de EAS, no en Expo Go.</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2/1/1</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr">
         <is>
-          <t>1/1/0,5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M32" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2/1/1</t>
         </is>
       </c>
       <c r="N32" s="6" t="inlineStr">
         <is>
-          <t>1/1/0,5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
-          <t>1/0,5/0,5</t>
+          <t>2/1/0,5</t>
         </is>
       </c>
       <c r="P32" s="6" t="inlineStr">
@@ -3659,7 +3659,7 @@
       </c>
       <c r="Q32" s="6" t="inlineStr">
         <is>
-          <t>RF-029, RF-031</t>
+          <t>RF-025</t>
         </is>
       </c>
       <c r="R32" s="6" t="inlineStr">
@@ -3669,12 +3669,12 @@
       </c>
       <c r="S32" s="4" t="inlineStr">
         <is>
-          <t>HU21</t>
+          <t>HU19</t>
         </is>
       </c>
       <c r="T32" s="4" t="inlineStr">
         <is>
-          <t>Jest useUsuarioStore, empresas</t>
+          <t>TC-PUSH-01..05; Jest notificaciones</t>
         </is>
       </c>
       <c r="U32" s="6" t="inlineStr">
@@ -3696,17 +3696,17 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>RF-031</t>
+          <t>RF-029</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Equipo e invitaciones</t>
+          <t>Alta de empresa</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>El propietario o un administrador invita por un enlace que abre la app (o la página web) con el código; asigna roles y puede quitar miembros.</t>
+          <t>Un usuario crea su empresa con nombre, CUIT y un enlace propio de tienda.</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -3718,14 +3718,14 @@
         <v>46318</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>46322</v>
+        <v>46318</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: HU21. Página docs/invitacion en GitHub Pages.</t>
+          <t>Etapa 1: HU21. Migración 06.</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
@@ -3735,24 +3735,24 @@
       </c>
       <c r="L33" s="6" t="inlineStr">
         <is>
+          <t>1/1/0,5</t>
+        </is>
+      </c>
+      <c r="M33" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N33" s="6" t="inlineStr">
+        <is>
           <t>2/1/1</t>
         </is>
       </c>
-      <c r="M33" s="6" t="inlineStr">
+      <c r="O33" s="6" t="inlineStr">
         <is>
           <t>1/0,5/0,5</t>
         </is>
       </c>
-      <c r="N33" s="6" t="inlineStr">
-        <is>
-          <t>1/1/0,5</t>
-        </is>
-      </c>
-      <c r="O33" s="6" t="inlineStr">
-        <is>
-          <t>1/1/0,5</t>
-        </is>
-      </c>
       <c r="P33" s="6" t="inlineStr">
         <is>
           <t>—</t>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="Q33" s="6" t="inlineStr">
         <is>
-          <t>RF-029</t>
+          <t>RF-002</t>
         </is>
       </c>
       <c r="R33" s="6" t="inlineStr">
@@ -3797,17 +3797,17 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>RF-032</t>
+          <t>RF-030</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Sedes</t>
+          <t>Modo Yo / Empresa</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>La empresa carga sus sedes con dirección; el stock y el retiro se asocian a una sede.</t>
+          <t>Un empleado elige si vende como particular o como la empresa; el propietario vende sólo como empresa; al invitarlo, el empleado queda en modo empresa.</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -3819,14 +3819,14 @@
         <v>46318</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>46318</v>
+        <v>46322</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: HU21. Migración 08.</t>
+          <t>Etapa 1: HU21. Migraciones 15 y 16.</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -3846,14 +3846,14 @@
       </c>
       <c r="N34" s="6" t="inlineStr">
         <is>
+          <t>1/1/0,5</t>
+        </is>
+      </c>
+      <c r="O34" s="6" t="inlineStr">
+        <is>
           <t>1/0,5/0,5</t>
         </is>
       </c>
-      <c r="O34" s="6" t="inlineStr">
-        <is>
-          <t>1/0,5/0,5</t>
-        </is>
-      </c>
       <c r="P34" s="6" t="inlineStr">
         <is>
           <t>—</t>
@@ -3861,12 +3861,12 @@
       </c>
       <c r="Q34" s="6" t="inlineStr">
         <is>
-          <t>RF-029</t>
+          <t>RF-029, RF-031</t>
         </is>
       </c>
       <c r="R34" s="6" t="inlineStr">
         <is>
-          <t>RF-024</t>
+          <t>—</t>
         </is>
       </c>
       <c r="S34" s="4" t="inlineStr">
@@ -3876,7 +3876,7 @@
       </c>
       <c r="T34" s="4" t="inlineStr">
         <is>
-          <t>Jest empresas</t>
+          <t>Jest useUsuarioStore, empresas</t>
         </is>
       </c>
       <c r="U34" s="6" t="inlineStr">
@@ -3898,61 +3898,61 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>RF-033</t>
+          <t>RF-031</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Tienda pública de la empresa</t>
+          <t>Equipo e invitaciones</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Cada empresa tiene una tienda con sus prendas en /tienda/&lt;enlace&gt;.</t>
+          <t>El propietario o un administrador invita por un enlace que abre la app (o la página web) con el código; asigna roles y puede quitar miembros.</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Frontend / Backend / Base de Datos</t>
         </is>
       </c>
       <c r="G35" s="5" t="n">
         <v>46318</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>46318</v>
+        <v>46322</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: HU21.</t>
+          <t>Etapa 1: HU21. Página docs/invitacion en GitHub Pages.</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr">
         <is>
+          <t>2/1/1</t>
+        </is>
+      </c>
+      <c r="M35" s="6" t="inlineStr">
+        <is>
+          <t>1/0,5/0,5</t>
+        </is>
+      </c>
+      <c r="N35" s="6" t="inlineStr">
+        <is>
           <t>1/1/0,5</t>
         </is>
       </c>
-      <c r="M35" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N35" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
-          <t>1/0,5/0,5</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="P35" s="6" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="Q35" s="6" t="inlineStr">
         <is>
-          <t>RF-029, RF-016</t>
+          <t>RF-029</t>
         </is>
       </c>
       <c r="R35" s="6" t="inlineStr">
@@ -3977,7 +3977,7 @@
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>Planilla QA (manual)</t>
+          <t>Jest empresas</t>
         </is>
       </c>
       <c r="U35" s="6" t="inlineStr">
@@ -3999,17 +3999,17 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>RF-034</t>
+          <t>RF-032</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Métricas de ventas</t>
+          <t>Sedes</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>La empresa ve ventas, unidades e ingresos de hoy, esta semana, este mes o un rango personalizado de hasta un año.</t>
+          <t>La empresa carga sus sedes con dirección; el stock y el retiro se asocian a una sede.</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -4021,14 +4021,14 @@
         <v>46318</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>46322</v>
+        <v>46318</v>
       </c>
       <c r="I36" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: HU21, Could C1. Migraciones 11 y 17.</t>
+          <t>Etapa 1: HU21. Migración 08.</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L36" s="6" t="inlineStr">
         <is>
-          <t>2/1/1</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="M36" s="6" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="N36" s="6" t="inlineStr">
         <is>
-          <t>1/1/0,5</t>
+          <t>1/0,5/0,5</t>
         </is>
       </c>
       <c r="O36" s="6" t="inlineStr">
@@ -4063,12 +4063,12 @@
       </c>
       <c r="Q36" s="6" t="inlineStr">
         <is>
-          <t>RF-025, RF-029</t>
+          <t>RF-029</t>
         </is>
       </c>
       <c r="R36" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RF-024</t>
         </is>
       </c>
       <c r="S36" s="4" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="T36" s="4" t="inlineStr">
         <is>
-          <t>Jest rangoFechas, pedidos</t>
+          <t>Jest empresas</t>
         </is>
       </c>
       <c r="U36" s="6" t="inlineStr">
@@ -4095,27 +4095,27 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Administración</t>
+          <t>Modo empresa</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>RF-035</t>
+          <t>RF-033</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Panel de administración</t>
+          <t>Tienda pública de la empresa</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Un administrador de la plataforma ve usuarios, empresas y publicaciones y puede dar de baja contenido.</t>
+          <t>Cada empresa tiene una tienda con sus prendas en /tienda/&lt;enlace&gt;.</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Frontend / Base de Datos</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="G37" s="5" t="n">
@@ -4129,7 +4129,7 @@
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>Migración 07. Sin HU en Etapa 1 (pendiente de agregar).</t>
+          <t>Etapa 1: HU21.</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -4149,7 +4149,7 @@
       </c>
       <c r="N37" s="6" t="inlineStr">
         <is>
-          <t>1/1/0,5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O37" s="6" t="inlineStr">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="Q37" s="6" t="inlineStr">
         <is>
-          <t>RF-003</t>
+          <t>RF-029, RF-016</t>
         </is>
       </c>
       <c r="R37" s="6" t="inlineStr">
@@ -4174,7 +4174,7 @@
       </c>
       <c r="S37" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>HU21</t>
         </is>
       </c>
       <c r="T37" s="4" t="inlineStr">
@@ -4196,22 +4196,22 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Configuración</t>
+          <t>Modo empresa</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>RF-036</t>
+          <t>RF-034</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Ajustes guardados</t>
+          <t>Métricas de ventas</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Los interruptores de notificaciones, correos y promociones se guardan en el perfil y se respetan.</t>
+          <t>La empresa ve ventas, unidades e ingresos de hoy, esta semana, este mes o un rango personalizado de hasta un año.</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -4220,17 +4220,17 @@
         </is>
       </c>
       <c r="G38" s="5" t="n">
-        <v>46279</v>
+        <v>46318</v>
       </c>
       <c r="H38" s="5" t="n">
         <v>46322</v>
       </c>
       <c r="I38" s="6" t="n">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: HU19.</t>
+          <t>Etapa 1: HU21, Could C1. Migraciones 11 y 17.</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -4240,24 +4240,24 @@
       </c>
       <c r="L38" s="6" t="inlineStr">
         <is>
+          <t>2/1/1</t>
+        </is>
+      </c>
+      <c r="M38" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N38" s="6" t="inlineStr">
+        <is>
           <t>1/1/0,5</t>
         </is>
       </c>
-      <c r="M38" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N38" s="6" t="inlineStr">
+      <c r="O38" s="6" t="inlineStr">
         <is>
           <t>1/0,5/0,5</t>
         </is>
       </c>
-      <c r="O38" s="6" t="inlineStr">
-        <is>
-          <t>1/0,5/0,5</t>
-        </is>
-      </c>
       <c r="P38" s="6" t="inlineStr">
         <is>
           <t>—</t>
@@ -4265,7 +4265,7 @@
       </c>
       <c r="Q38" s="6" t="inlineStr">
         <is>
-          <t>RF-005</t>
+          <t>RF-025, RF-029</t>
         </is>
       </c>
       <c r="R38" s="6" t="inlineStr">
@@ -4275,12 +4275,12 @@
       </c>
       <c r="S38" s="4" t="inlineStr">
         <is>
-          <t>HU19</t>
+          <t>HU21</t>
         </is>
       </c>
       <c r="T38" s="4" t="inlineStr">
         <is>
-          <t>Planilla QA (manual)</t>
+          <t>Jest rangoFechas, pedidos</t>
         </is>
       </c>
       <c r="U38" s="6" t="inlineStr">
@@ -4297,41 +4297,41 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Configuración</t>
+          <t>Administración</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>RF-037</t>
+          <t>RF-035</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Modo oscuro</t>
+          <t>Panel de administración</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Desde Ajustes &gt; Apariencia el usuario activa el modo oscuro; la preferencia queda guardada en el dispositivo.</t>
+          <t>Un administrador de la plataforma verifica las empresas nuevas, las suspende con un motivo que la empresa ve y las reactiva; sólo los administradores entran al panel.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Frontend / Base de Datos</t>
         </is>
       </c>
       <c r="G39" s="5" t="n">
-        <v>46322</v>
+        <v>46318</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>46322</v>
+        <v>46318</v>
       </c>
       <c r="I39" s="6" t="n">
         <v>1</v>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: HU19, RNF2 (tokens en constants/theme.ts).</t>
+          <t>Etapa 1: HU27. Migración 07.</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="L39" s="6" t="inlineStr">
         <is>
-          <t>2/1/1</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="M39" s="6" t="inlineStr">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="N39" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="O39" s="6" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="Q39" s="6" t="inlineStr">
         <is>
-          <t>RF-036</t>
+          <t>RF-003</t>
         </is>
       </c>
       <c r="R39" s="6" t="inlineStr">
@@ -4376,7 +4376,7 @@
       </c>
       <c r="S39" s="4" t="inlineStr">
         <is>
-          <t>HU19</t>
+          <t>HU27</t>
         </is>
       </c>
       <c r="T39" s="4" t="inlineStr">
@@ -4398,41 +4398,41 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Conectividad</t>
+          <t>Configuración</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>RF-038</t>
+          <t>RF-036</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Aviso sin conexión</t>
+          <t>Ajustes guardados</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Sin Internet se muestra un aviso fijo y las acciones que necesitan red se bloquean con un mensaje claro.</t>
+          <t>Los interruptores de notificaciones, correos y promociones se guardan en el perfil y se respetan.</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Frontend / Base de Datos</t>
         </is>
       </c>
       <c r="G40" s="5" t="n">
-        <v>46313</v>
+        <v>46279</v>
       </c>
       <c r="H40" s="5" t="n">
         <v>46322</v>
       </c>
       <c r="I40" s="6" t="n">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: HU16. NetInfo.</t>
+          <t>Etapa 1: HU19.</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -4452,7 +4452,7 @@
       </c>
       <c r="N40" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1/0,5/0,5</t>
         </is>
       </c>
       <c r="O40" s="6" t="inlineStr">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="Q40" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RF-005</t>
         </is>
       </c>
       <c r="R40" s="6" t="inlineStr">
@@ -4477,12 +4477,12 @@
       </c>
       <c r="S40" s="4" t="inlineStr">
         <is>
-          <t>HU16</t>
+          <t>HU19</t>
         </is>
       </c>
       <c r="T40" s="4" t="inlineStr">
         <is>
-          <t>TC-HU16-01 (manual, modo avión)</t>
+          <t>Planilla QA (manual)</t>
         </is>
       </c>
       <c r="U40" s="6" t="inlineStr">
@@ -4492,143 +4492,149 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>RF</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Seguridad</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>RF-039</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Chat interno</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Comprador y vendedor se comunican por un chat dentro de la app sin compartir teléfono ni correo.</t>
-        </is>
-      </c>
-      <c r="F41" s="8" t="inlineStr">
-        <is>
-          <t>Frontend / Backend / Base de Datos</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="n"/>
-      <c r="H41" s="7" t="n"/>
-      <c r="I41" s="7" t="n"/>
-      <c r="J41" s="8" t="inlineStr">
-        <is>
-          <t>Etapa 1: HU15. Segunda entrega, pendiente.</t>
-        </is>
-      </c>
-      <c r="K41" s="7" t="inlineStr">
-        <is>
-          <t>5/3/2</t>
-        </is>
-      </c>
-      <c r="L41" s="7" t="inlineStr">
-        <is>
-          <t>5/3/2</t>
-        </is>
-      </c>
-      <c r="M41" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N41" s="7" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Configuración</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>RF-037</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Modo oscuro</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Desde Ajustes &gt; Apariencia el usuario activa el modo oscuro; la preferencia queda guardada en el dispositivo.</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="n">
+        <v>46322</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <v>46322</v>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Etapa 1: HU19, RNF2 (tokens en constants/theme.ts).</t>
+        </is>
+      </c>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L41" s="6" t="inlineStr">
         <is>
           <t>2/1/1</t>
         </is>
       </c>
-      <c r="O41" s="7" t="inlineStr">
-        <is>
-          <t>2/1/1</t>
-        </is>
-      </c>
-      <c r="P41" s="7" t="inlineStr">
-        <is>
-          <t>1/1/0,5</t>
-        </is>
-      </c>
-      <c r="Q41" s="7" t="inlineStr">
-        <is>
-          <t>RF-021</t>
-        </is>
-      </c>
-      <c r="R41" s="7" t="inlineStr">
-        <is>
-          <t>RF-028</t>
-        </is>
-      </c>
-      <c r="S41" s="8" t="inlineStr">
-        <is>
-          <t>HU15</t>
-        </is>
-      </c>
-      <c r="T41" s="8" t="inlineStr">
-        <is>
-          <t>Sin casos todavía</t>
-        </is>
-      </c>
-      <c r="U41" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="M41" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N41" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O41" s="6" t="inlineStr">
+        <is>
+          <t>1/0,5/0,5</t>
+        </is>
+      </c>
+      <c r="P41" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q41" s="6" t="inlineStr">
+        <is>
+          <t>RF-036</t>
+        </is>
+      </c>
+      <c r="R41" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S41" s="4" t="inlineStr">
+        <is>
+          <t>HU19</t>
+        </is>
+      </c>
+      <c r="T41" s="4" t="inlineStr">
+        <is>
+          <t>Planilla QA (manual)</t>
+        </is>
+      </c>
+      <c r="U41" s="6" t="inlineStr">
+        <is>
+          <t>Implementado</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>RNF</t>
+          <t>RF</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>No funcional</t>
+          <t>Conectividad</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>RNF-001</t>
+          <t>RF-038</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Rendimiento del catálogo</t>
+          <t>Aviso sin conexión</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Las consultas del catálogo responden en menos de 1,5 segundos con red móvil estándar.</t>
+          <t>Sin Internet se muestra un aviso fijo y las acciones que necesitan red se bloquean con un mensaje claro.</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Backend / Testing</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="G42" s="5" t="n">
-        <v>46319</v>
+        <v>46313</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="I42" s="6" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: RNF1. ISO 25010: eficiencia de desempeño.</t>
+          <t>Etapa 1: HU16. NetInfo.</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
@@ -4638,7 +4644,7 @@
       </c>
       <c r="L42" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="M42" s="6" t="inlineStr">
@@ -4653,138 +4659,132 @@
       </c>
       <c r="O42" s="6" t="inlineStr">
         <is>
+          <t>1/0,5/0,5</t>
+        </is>
+      </c>
+      <c r="P42" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q42" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R42" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S42" s="4" t="inlineStr">
+        <is>
+          <t>HU16</t>
+        </is>
+      </c>
+      <c r="T42" s="4" t="inlineStr">
+        <is>
+          <t>TC-HU16-01 (manual, modo avión)</t>
+        </is>
+      </c>
+      <c r="U42" s="6" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>RF-039</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Chat interno</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Comprador y vendedor se comunican por un chat dentro de la app sin compartir teléfono ni correo.</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Frontend / Backend / Base de Datos</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="n"/>
+      <c r="H43" s="7" t="n"/>
+      <c r="I43" s="7" t="n"/>
+      <c r="J43" s="8" t="inlineStr">
+        <is>
+          <t>Etapa 1: HU15. Segunda entrega, pendiente.</t>
+        </is>
+      </c>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>5/3/2</t>
+        </is>
+      </c>
+      <c r="L43" s="7" t="inlineStr">
+        <is>
+          <t>5/3/2</t>
+        </is>
+      </c>
+      <c r="M43" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N43" s="7" t="inlineStr">
+        <is>
+          <t>2/1/1</t>
+        </is>
+      </c>
+      <c r="O43" s="7" t="inlineStr">
+        <is>
+          <t>2/1/1</t>
+        </is>
+      </c>
+      <c r="P43" s="7" t="inlineStr">
+        <is>
           <t>1/1/0,5</t>
         </is>
       </c>
-      <c r="P42" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q42" s="6" t="inlineStr">
-        <is>
-          <t>RF-007</t>
-        </is>
-      </c>
-      <c r="R42" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S42" s="4" t="inlineStr">
-        <is>
-          <t>HU03</t>
-        </is>
-      </c>
-      <c r="T42" s="4" t="inlineStr">
-        <is>
-          <t>JMeter catalogo.jmx; Postman performance</t>
-        </is>
-      </c>
-      <c r="U42" s="6" t="inlineStr">
-        <is>
-          <t>Implementado</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>RNF</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>No funcional</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>RNF-002</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Tokens de diseño</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>Todos los estilos usan los tokens de constants/theme.ts (colores, espacios, radios, tipografía), con paleta clara y oscura.</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="n">
-        <v>46249</v>
-      </c>
-      <c r="H43" s="5" t="n">
-        <v>46322</v>
-      </c>
-      <c r="I43" s="6" t="n">
-        <v>74</v>
-      </c>
-      <c r="J43" s="4" t="inlineStr">
-        <is>
-          <t>Etapa 1: RNF2. ISO 25010: mantenibilidad.</t>
-        </is>
-      </c>
-      <c r="K43" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L43" s="6" t="inlineStr">
-        <is>
-          <t>1/1/0,5</t>
-        </is>
-      </c>
-      <c r="M43" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N43" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O43" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P43" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q43" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R43" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S43" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="T43" s="4" t="inlineStr">
-        <is>
-          <t>Revisión de código (checklist peer review)</t>
-        </is>
-      </c>
-      <c r="U43" s="6" t="inlineStr">
-        <is>
-          <t>Implementado</t>
+      <c r="Q43" s="7" t="inlineStr">
+        <is>
+          <t>RF-021</t>
+        </is>
+      </c>
+      <c r="R43" s="7" t="inlineStr">
+        <is>
+          <t>RF-028</t>
+        </is>
+      </c>
+      <c r="S43" s="8" t="inlineStr">
+        <is>
+          <t>HU15</t>
+        </is>
+      </c>
+      <c r="T43" s="8" t="inlineStr">
+        <is>
+          <t>Sin casos todavía</t>
+        </is>
+      </c>
+      <c r="U43" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -4801,36 +4801,36 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>RNF-003</t>
+          <t>RNF-001</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Seguridad a nivel de fila (RLS)</t>
+          <t>Rendimiento del catálogo</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Cada usuario sólo puede modificar o borrar sus propios datos; las políticas están versionadas en supabase/migraciones.</t>
+          <t>Las consultas del catálogo responden en menos de 1,5 segundos con red móvil estándar.</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Base de Datos</t>
+          <t>Backend / Testing</t>
         </is>
       </c>
       <c r="G44" s="5" t="n">
-        <v>46313</v>
+        <v>46319</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>46322</v>
+        <v>46319</v>
       </c>
       <c r="I44" s="6" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: RNF3. ISO 25010: seguridad.</t>
+          <t>Etapa 1: RNF1. ISO 25010: eficiencia de desempeño.</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="N44" s="6" t="inlineStr">
         <is>
-          <t>2/1/1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O44" s="6" t="inlineStr">
@@ -4865,7 +4865,7 @@
       </c>
       <c r="Q44" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RF-007</t>
         </is>
       </c>
       <c r="R44" s="6" t="inlineStr">
@@ -4875,12 +4875,12 @@
       </c>
       <c r="S44" s="4" t="inlineStr">
         <is>
-          <t>HU08</t>
+          <t>HU03</t>
         </is>
       </c>
       <c r="T44" s="4" t="inlineStr">
         <is>
-          <t>Postman negativos/editar ajeno</t>
+          <t>JMeter catalogo.jmx; Postman performance</t>
         </is>
       </c>
       <c r="U44" s="6" t="inlineStr">
@@ -4902,36 +4902,36 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>RNF-004</t>
+          <t>RNF-002</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Confidencialidad de datos personales</t>
+          <t>Tokens de diseño</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Los endpoints públicos no exponen correo, teléfono ni dirección de los vendedores particulares.</t>
+          <t>Todos los estilos usan los tokens de constants/theme.ts (colores, espacios, radios, tipografía), con paleta clara y oscura.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Base de Datos</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="G45" s="5" t="n">
-        <v>46322</v>
+        <v>46249</v>
       </c>
       <c r="H45" s="5" t="n">
         <v>46322</v>
       </c>
       <c r="I45" s="6" t="n">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>Etapa 1: RNF4. Vistas públicas (migración 15).</t>
+          <t>Etapa 1: RNF2. ISO 25010: mantenibilidad.</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="L45" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="M45" s="6" t="inlineStr">
@@ -4951,12 +4951,12 @@
       </c>
       <c r="N45" s="6" t="inlineStr">
         <is>
-          <t>1/0,5/0,5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O45" s="6" t="inlineStr">
         <is>
-          <t>1/0,5/0,5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="P45" s="6" t="inlineStr">
@@ -4966,7 +4966,7 @@
       </c>
       <c r="Q45" s="6" t="inlineStr">
         <is>
-          <t>RNF-003</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R45" s="6" t="inlineStr">
@@ -4981,7 +4981,7 @@
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>Postman negativos</t>
+          <t>Revisión de código (checklist peer review)</t>
         </is>
       </c>
       <c r="U45" s="6" t="inlineStr">
@@ -5003,36 +5003,36 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>RNF-005</t>
+          <t>RNF-003</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Sesión cifrada</t>
+          <t>Seguridad a nivel de fila (RLS)</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Los tokens de sesión se guardan cifrados (SecureStore) y nunca en texto plano.</t>
+          <t>Cada usuario sólo puede modificar o borrar sus propios datos; las políticas están versionadas en supabase/migraciones.</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Base de Datos</t>
         </is>
       </c>
       <c r="G46" s="5" t="n">
-        <v>46319</v>
+        <v>46313</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="I46" s="6" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t>ISO 25010: seguridad.</t>
+          <t>Etapa 1: RNF3. ISO 25010: seguridad.</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
@@ -5042,7 +5042,7 @@
       </c>
       <c r="L46" s="6" t="inlineStr">
         <is>
-          <t>1/0,5/0,5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M46" s="6" t="inlineStr">
@@ -5052,12 +5052,12 @@
       </c>
       <c r="N46" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2/1/1</t>
         </is>
       </c>
       <c r="O46" s="6" t="inlineStr">
         <is>
-          <t>1/0,5/0,5</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="P46" s="6" t="inlineStr">
@@ -5077,12 +5077,12 @@
       </c>
       <c r="S46" s="4" t="inlineStr">
         <is>
-          <t>HU02</t>
+          <t>HU08</t>
         </is>
       </c>
       <c r="T46" s="4" t="inlineStr">
         <is>
-          <t>Jest secureSessionStorage</t>
+          <t>Postman negativos/editar ajeno</t>
         </is>
       </c>
       <c r="U46" s="6" t="inlineStr">
@@ -5104,22 +5104,22 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>RNF-006</t>
+          <t>RNF-004</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Mensajes en español</t>
+          <t>Confidencialidad de datos personales</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Todos los errores, incluidos los de Supabase Auth y la base, se muestran en español y sin detalles técnicos.</t>
+          <t>Los endpoints públicos no exponen correo, teléfono ni dirección de los vendedores particulares.</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Base de Datos</t>
         </is>
       </c>
       <c r="G47" s="5" t="n">
@@ -5133,7 +5133,7 @@
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>ISO 25010: usabilidad.</t>
+          <t>Etapa 1: RNF4. Vistas públicas (migración 15).</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="L47" s="6" t="inlineStr">
         <is>
-          <t>1/1/0,5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M47" s="6" t="inlineStr">
@@ -5153,7 +5153,7 @@
       </c>
       <c r="N47" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1/0,5/0,5</t>
         </is>
       </c>
       <c r="O47" s="6" t="inlineStr">
@@ -5168,7 +5168,7 @@
       </c>
       <c r="Q47" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RNF-003</t>
         </is>
       </c>
       <c r="R47" s="6" t="inlineStr">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="T47" s="4" t="inlineStr">
         <is>
-          <t>Jest erroresSupabase</t>
+          <t>Postman negativos</t>
         </is>
       </c>
       <c r="U47" s="6" t="inlineStr">
@@ -5205,36 +5205,36 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>RNF-007</t>
+          <t>RNF-005</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Consistencia de la compra</t>
+          <t>Sesión cifrada</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>La compra se confirma en una única transacción en el servidor y es idempotente.</t>
+          <t>Los tokens de sesión se guardan cifrados (SecureStore) y nunca en texto plano.</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Backend / Base de Datos</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="G48" s="5" t="n">
-        <v>46313</v>
+        <v>46319</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>46313</v>
+        <v>46319</v>
       </c>
       <c r="I48" s="6" t="n">
         <v>1</v>
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>ISO 25010: fiabilidad.</t>
+          <t>ISO 25010: seguridad.</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
@@ -5244,7 +5244,7 @@
       </c>
       <c r="L48" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1/0,5/0,5</t>
         </is>
       </c>
       <c r="M48" s="6" t="inlineStr">
@@ -5254,12 +5254,12 @@
       </c>
       <c r="N48" s="6" t="inlineStr">
         <is>
-          <t>1/1/0,5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O48" s="6" t="inlineStr">
         <is>
-          <t>1/1/0,5</t>
+          <t>1/0,5/0,5</t>
         </is>
       </c>
       <c r="P48" s="6" t="inlineStr">
@@ -5279,12 +5279,12 @@
       </c>
       <c r="S48" s="4" t="inlineStr">
         <is>
-          <t>HU14</t>
+          <t>HU02</t>
         </is>
       </c>
       <c r="T48" s="4" t="inlineStr">
         <is>
-          <t>TC-HU14-02; Postman concurrencia</t>
+          <t>Jest secureSessionStorage</t>
         </is>
       </c>
       <c r="U48" s="6" t="inlineStr">
@@ -5306,36 +5306,36 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>RNF-008</t>
+          <t>RNF-006</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Integración continua</t>
+          <t>Mensajes en español</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Cada push y PR corre tipos, lint y tests en GitHub Actions; no se mergea en rojo.</t>
+          <t>Todos los errores, incluidos los de Supabase Auth y la base, se muestran en español y sin detalles técnicos.</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Implementación / Testing</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="G49" s="5" t="n">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="H49" s="5" t="n">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="I49" s="6" t="n">
         <v>1</v>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>.github/workflows/test.yml.</t>
+          <t>ISO 25010: usabilidad.</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
@@ -5345,24 +5345,24 @@
       </c>
       <c r="L49" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1/1/0,5</t>
         </is>
       </c>
       <c r="M49" s="6" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N49" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O49" s="6" t="inlineStr">
+        <is>
           <t>1/0,5/0,5</t>
         </is>
       </c>
-      <c r="N49" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O49" s="6" t="inlineStr">
-        <is>
-          <t>1/0,5/0,5</t>
-        </is>
-      </c>
       <c r="P49" s="6" t="inlineStr">
         <is>
           <t>—</t>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="T49" s="4" t="inlineStr">
         <is>
-          <t>GitHub Actions</t>
+          <t>Jest erroresSupabase</t>
         </is>
       </c>
       <c r="U49" s="6" t="inlineStr">
@@ -5407,103 +5407,305 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>RNF-009</t>
+          <t>RNF-007</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Accesibilidad</t>
+          <t>Consistencia de la compra</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Los controles tienen etiquetas accesibles y testID para pruebas automáticas.</t>
+          <t>La compra se confirma en una única transacción en el servidor y es idempotente.</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend / Base de Datos</t>
         </is>
       </c>
       <c r="G50" s="5" t="n">
-        <v>46319</v>
+        <v>46313</v>
       </c>
       <c r="H50" s="5" t="n">
-        <v>46319</v>
+        <v>46313</v>
       </c>
       <c r="I50" s="6" t="n">
         <v>1</v>
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
+          <t>ISO 25010: fiabilidad.</t>
+        </is>
+      </c>
+      <c r="K50" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L50" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M50" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N50" s="6" t="inlineStr">
+        <is>
+          <t>1/1/0,5</t>
+        </is>
+      </c>
+      <c r="O50" s="6" t="inlineStr">
+        <is>
+          <t>1/1/0,5</t>
+        </is>
+      </c>
+      <c r="P50" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q50" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R50" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S50" s="4" t="inlineStr">
+        <is>
+          <t>HU14</t>
+        </is>
+      </c>
+      <c r="T50" s="4" t="inlineStr">
+        <is>
+          <t>TC-HU14-02; Postman concurrencia</t>
+        </is>
+      </c>
+      <c r="U50" s="6" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>RNF</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>No funcional</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>RNF-008</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Integración continua</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>Cada push y PR corre tipos, lint y tests en GitHub Actions; no se mergea en rojo.</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Implementación / Testing</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="n">
+        <v>46319</v>
+      </c>
+      <c r="H51" s="5" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>.github/workflows/test.yml.</t>
+        </is>
+      </c>
+      <c r="K51" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L51" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M51" s="6" t="inlineStr">
+        <is>
+          <t>1/0,5/0,5</t>
+        </is>
+      </c>
+      <c r="N51" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O51" s="6" t="inlineStr">
+        <is>
+          <t>1/0,5/0,5</t>
+        </is>
+      </c>
+      <c r="P51" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q51" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R51" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S51" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T51" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Actions</t>
+        </is>
+      </c>
+      <c r="U51" s="6" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>RNF</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>No funcional</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>RNF-009</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Accesibilidad</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Los controles tienen etiquetas accesibles y testID para pruebas automáticas.</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="n">
+        <v>46319</v>
+      </c>
+      <c r="H52" s="5" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I52" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
           <t>ISO 25010: usabilidad.</t>
         </is>
       </c>
-      <c r="K50" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L50" s="6" t="inlineStr">
+      <c r="K52" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L52" s="6" t="inlineStr">
         <is>
           <t>1/1/0,5</t>
         </is>
       </c>
-      <c r="M50" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N50" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O50" s="6" t="inlineStr">
+      <c r="M52" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N52" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O52" s="6" t="inlineStr">
         <is>
           <t>1/0,5/0,5</t>
         </is>
       </c>
-      <c r="P50" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q50" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R50" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S50" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="T50" s="4" t="inlineStr">
+      <c r="P52" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q52" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R52" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S52" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T52" s="4" t="inlineStr">
         <is>
           <t>Maestro (.maestro)</t>
         </is>
       </c>
-      <c r="U50" s="6" t="inlineStr">
+      <c r="U52" s="6" t="inlineStr">
         <is>
           <t>Implementado</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:U50"/>
+  <autoFilter ref="A2:U52"/>
   <mergeCells count="3">
     <mergeCell ref="K1:P1"/>
     <mergeCell ref="S1:U1"/>
     <mergeCell ref="Q1:R1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="U3:U50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U3:U52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Implementado,Parcial,Pendiente"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5517,7 +5719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6027,7 +6229,7 @@
         <v>10.33</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>1.58</v>
+        <v>0.25</v>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
@@ -6555,7 +6757,7 @@
         <v>13.5</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>1.58</v>
+        <v>0.25</v>
       </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
@@ -6619,17 +6821,17 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Medio de pago simulado</t>
+          <t>Medios de pago</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F24" s="6">
         <f>ROUND((C24+4*D24+E24)/6,2)</f>
@@ -6648,10 +6850,10 @@
         <v>13.5</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>14.67</v>
+        <v>19.58</v>
       </c>
       <c r="K24" s="6" t="n">
-        <v>5.17</v>
+        <v>0.25</v>
       </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
@@ -6758,22 +6960,22 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>RF-023</t>
+          <t>RF-040</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Historial de compras</t>
+          <t>Comisión y cuotas con tarjeta de crédito</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F27" s="6">
         <f>ROUND((C27+4*D27+E27)/6,2)</f>
@@ -6785,17 +6987,17 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>RF-021</t>
+          <t>RF-020, RF-021</t>
         </is>
       </c>
       <c r="I27" s="6" t="n">
         <v>26.5</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>28.83</v>
+        <v>30.17</v>
       </c>
       <c r="K27" s="6" t="n">
-        <v>7.25</v>
+        <v>5.92</v>
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
@@ -6806,22 +7008,22 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>RF-024</t>
+          <t>RF-041</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Geolocalización y mapa</t>
+          <t>Pago con Mercado Pago</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F28" s="6">
         <f>ROUND((C28+4*D28+E28)/6,2)</f>
@@ -6833,17 +7035,17 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RF-020, RF-021</t>
         </is>
       </c>
       <c r="I28" s="6" t="n">
-        <v>0</v>
+        <v>26.5</v>
       </c>
       <c r="J28" s="6" t="n">
-        <v>4.08</v>
+        <v>31.83</v>
       </c>
       <c r="K28" s="6" t="n">
-        <v>32</v>
+        <v>4.25</v>
       </c>
       <c r="L28" s="6" t="inlineStr">
         <is>
@@ -6854,22 +7056,22 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>RF-025</t>
+          <t>RF-023</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Mis ventas y estado de pedidos</t>
+          <t>Historial de compras</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="6" t="n">
         <v>4</v>
-      </c>
-      <c r="E29" s="6" t="n">
-        <v>6</v>
       </c>
       <c r="F29" s="6">
         <f>ROUND((C29+4*D29+E29)/6,2)</f>
@@ -6888,10 +7090,10 @@
         <v>26.5</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>30.67</v>
+        <v>28.83</v>
       </c>
       <c r="K29" s="6" t="n">
-        <v>1.25</v>
+        <v>7.25</v>
       </c>
       <c r="L29" s="6" t="inlineStr">
         <is>
@@ -6902,22 +7104,22 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>RF-026</t>
+          <t>RF-024</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Calificación de vendedores</t>
+          <t>Geolocalización y mapa</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F30" s="6">
         <f>ROUND((C30+4*D30+E30)/6,2)</f>
@@ -6929,17 +7131,17 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>RF-025</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I30" s="6" t="n">
-        <v>30.67</v>
+        <v>0</v>
       </c>
       <c r="J30" s="6" t="n">
-        <v>32.75</v>
+        <v>4.08</v>
       </c>
       <c r="K30" s="6" t="n">
-        <v>1.25</v>
+        <v>32</v>
       </c>
       <c r="L30" s="6" t="inlineStr">
         <is>
@@ -6950,22 +7152,22 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>RF-027</t>
+          <t>RF-025</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Página pública del vendedor</t>
+          <t>Mis ventas y estado de pedidos</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F31" s="6">
         <f>ROUND((C31+4*D31+E31)/6,2)</f>
@@ -6977,14 +7179,14 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>RF-026</t>
+          <t>RF-021</t>
         </is>
       </c>
       <c r="I31" s="6" t="n">
-        <v>32.75</v>
+        <v>26.5</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>34.83</v>
+        <v>30.67</v>
       </c>
       <c r="K31" s="6" t="n">
         <v>1.25</v>
@@ -6998,22 +7200,22 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>RF-028</t>
+          <t>RF-026</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Notificaciones push</t>
+          <t>Calificación de vendedores</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="D32" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="6" t="n">
         <v>3</v>
-      </c>
-      <c r="E32" s="6" t="n">
-        <v>6</v>
       </c>
       <c r="F32" s="6">
         <f>ROUND((C32+4*D32+E32)/6,2)</f>
@@ -7032,10 +7234,10 @@
         <v>30.67</v>
       </c>
       <c r="J32" s="6" t="n">
-        <v>34.08</v>
+        <v>32.75</v>
       </c>
       <c r="K32" s="6" t="n">
-        <v>2</v>
+        <v>1.25</v>
       </c>
       <c r="L32" s="6" t="inlineStr">
         <is>
@@ -7046,22 +7248,22 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>RF-031</t>
+          <t>RF-027</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Equipo e invitaciones</t>
+          <t>Página pública del vendedor</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" s="6" t="n">
         <v>3</v>
-      </c>
-      <c r="D33" s="6" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="E33" s="6" t="n">
-        <v>6</v>
       </c>
       <c r="F33" s="6">
         <f>ROUND((C33+4*D33+E33)/6,2)</f>
@@ -7073,17 +7275,17 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>RF-029</t>
+          <t>RF-026</t>
         </is>
       </c>
       <c r="I33" s="6" t="n">
-        <v>12.83</v>
+        <v>32.75</v>
       </c>
       <c r="J33" s="6" t="n">
-        <v>17.33</v>
+        <v>34.83</v>
       </c>
       <c r="K33" s="6" t="n">
-        <v>16.33</v>
+        <v>1.25</v>
       </c>
       <c r="L33" s="6" t="inlineStr">
         <is>
@@ -7094,22 +7296,22 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>RF-030</t>
+          <t>RF-028</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Modo Yo / Empresa</t>
+          <t>Notificaciones push</t>
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F34" s="6">
         <f>ROUND((C34+4*D34+E34)/6,2)</f>
@@ -7121,17 +7323,17 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>RF-029, RF-031</t>
+          <t>RF-025</t>
         </is>
       </c>
       <c r="I34" s="6" t="n">
-        <v>17.33</v>
+        <v>30.67</v>
       </c>
       <c r="J34" s="6" t="n">
-        <v>19.75</v>
+        <v>34.08</v>
       </c>
       <c r="K34" s="6" t="n">
-        <v>16.33</v>
+        <v>2</v>
       </c>
       <c r="L34" s="6" t="inlineStr">
         <is>
@@ -7142,22 +7344,22 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>RF-033</t>
+          <t>RF-031</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Tienda pública de la empresa</t>
+          <t>Equipo e invitaciones</t>
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>1.5</v>
+        <v>4.5</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F35" s="6">
         <f>ROUND((C35+4*D35+E35)/6,2)</f>
@@ -7169,17 +7371,17 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>RF-029, RF-016</t>
+          <t>RF-029</t>
         </is>
       </c>
       <c r="I35" s="6" t="n">
-        <v>19.83</v>
+        <v>12.83</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>21.33</v>
+        <v>17.33</v>
       </c>
       <c r="K35" s="6" t="n">
-        <v>14.75</v>
+        <v>16.33</v>
       </c>
       <c r="L35" s="6" t="inlineStr">
         <is>
@@ -7190,22 +7392,22 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>RF-034</t>
+          <t>RF-030</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Métricas de ventas</t>
+          <t>Modo Yo / Empresa</t>
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D36" s="6" t="n">
         <v>2.5</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F36" s="6">
         <f>ROUND((C36+4*D36+E36)/6,2)</f>
@@ -7217,17 +7419,17 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>RF-025, RF-029</t>
+          <t>RF-029, RF-031</t>
         </is>
       </c>
       <c r="I36" s="6" t="n">
-        <v>30.67</v>
+        <v>17.33</v>
       </c>
       <c r="J36" s="6" t="n">
-        <v>33.33</v>
+        <v>19.75</v>
       </c>
       <c r="K36" s="6" t="n">
-        <v>2.75</v>
+        <v>16.33</v>
       </c>
       <c r="L36" s="6" t="inlineStr">
         <is>
@@ -7238,22 +7440,22 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>RF-035</t>
+          <t>RF-033</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Panel de administración</t>
+          <t>Tienda pública de la empresa</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="D37" s="6" t="n">
-        <v>2.5</v>
-      </c>
       <c r="E37" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37" s="6">
         <f>ROUND((C37+4*D37+E37)/6,2)</f>
@@ -7265,17 +7467,17 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>RF-003</t>
+          <t>RF-029, RF-016</t>
         </is>
       </c>
       <c r="I37" s="6" t="n">
-        <v>9</v>
+        <v>19.83</v>
       </c>
       <c r="J37" s="6" t="n">
-        <v>11.42</v>
+        <v>21.33</v>
       </c>
       <c r="K37" s="6" t="n">
-        <v>24.67</v>
+        <v>14.75</v>
       </c>
       <c r="L37" s="6" t="inlineStr">
         <is>
@@ -7286,22 +7488,22 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>RF-036</t>
+          <t>RF-034</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Ajustes guardados</t>
+          <t>Métricas de ventas</t>
         </is>
       </c>
       <c r="C38" s="6" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F38" s="6">
         <f>ROUND((C38+4*D38+E38)/6,2)</f>
@@ -7313,17 +7515,17 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>RF-005</t>
+          <t>RF-025, RF-029</t>
         </is>
       </c>
       <c r="I38" s="6" t="n">
-        <v>6.25</v>
+        <v>30.67</v>
       </c>
       <c r="J38" s="6" t="n">
-        <v>8.33</v>
+        <v>33.33</v>
       </c>
       <c r="K38" s="6" t="n">
-        <v>26</v>
+        <v>2.75</v>
       </c>
       <c r="L38" s="6" t="inlineStr">
         <is>
@@ -7334,19 +7536,19 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>RF-037</t>
+          <t>RF-035</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Modo oscuro</t>
+          <t>Panel de administración</t>
         </is>
       </c>
       <c r="C39" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="E39" s="6" t="n">
         <v>3</v>
@@ -7361,17 +7563,17 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>RF-036</t>
+          <t>RF-003</t>
         </is>
       </c>
       <c r="I39" s="6" t="n">
-        <v>8.33</v>
+        <v>9</v>
       </c>
       <c r="J39" s="6" t="n">
-        <v>10.08</v>
+        <v>11.42</v>
       </c>
       <c r="K39" s="6" t="n">
-        <v>26</v>
+        <v>24.67</v>
       </c>
       <c r="L39" s="6" t="inlineStr">
         <is>
@@ -7382,22 +7584,22 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>RF-038</t>
+          <t>RF-036</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Aviso sin conexión</t>
+          <t>Ajustes guardados</t>
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F40" s="6">
         <f>ROUND((C40+4*D40+E40)/6,2)</f>
@@ -7409,91 +7611,91 @@
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RF-005</t>
         </is>
       </c>
       <c r="I40" s="6" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
       <c r="J40" s="6" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="K40" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>RF-037</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Modo oscuro</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="K40" s="6" t="n">
-        <v>34.58</v>
-      </c>
-      <c r="L40" s="6" t="inlineStr">
+      <c r="D41" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" s="6">
+        <f>ROUND((C41+4*D41+E41)/6,2)</f>
+        <v/>
+      </c>
+      <c r="G41" s="6">
+        <f>ROUND((E41-C41)/6,2)</f>
+        <v/>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>RF-036</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="J41" s="6" t="n">
+        <v>10.08</v>
+      </c>
+      <c r="K41" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="L41" s="6" t="inlineStr">
         <is>
           <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>RF-039</t>
-        </is>
-      </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>Chat interno</t>
-        </is>
-      </c>
-      <c r="C41" s="11" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="D41" s="11" t="n">
-        <v>9</v>
-      </c>
-      <c r="E41" s="11" t="n">
-        <v>15</v>
-      </c>
-      <c r="F41" s="11">
-        <f>ROUND((C41+4*D41+E41)/6,2)</f>
-        <v/>
-      </c>
-      <c r="G41" s="11">
-        <f>ROUND((E41-C41)/6,2)</f>
-        <v/>
-      </c>
-      <c r="H41" s="11" t="inlineStr">
-        <is>
-          <t>RF-021</t>
-        </is>
-      </c>
-      <c r="I41" s="11" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="J41" s="11" t="n">
-        <v>36.08</v>
-      </c>
-      <c r="K41" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L41" s="11" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>RNF-001</t>
+          <t>RF-038</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Rendimiento del catálogo</t>
+          <t>Aviso sin conexión</t>
         </is>
       </c>
       <c r="C42" s="6" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F42" s="6">
         <f>ROUND((C42+4*D42+E42)/6,2)</f>
@@ -7505,17 +7707,17 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>RF-007</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I42" s="6" t="n">
-        <v>7.75</v>
+        <v>0</v>
       </c>
       <c r="J42" s="6" t="n">
-        <v>8.67</v>
+        <v>1.5</v>
       </c>
       <c r="K42" s="6" t="n">
-        <v>27.42</v>
+        <v>34.58</v>
       </c>
       <c r="L42" s="6" t="inlineStr">
         <is>
@@ -7524,72 +7726,72 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>RNF-002</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Tokens de diseño</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D43" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="6">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>RF-039</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>Chat interno</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D43" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="E43" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="F43" s="11">
         <f>ROUND((C43+4*D43+E43)/6,2)</f>
         <v/>
       </c>
-      <c r="G43" s="6">
+      <c r="G43" s="11">
         <f>ROUND((E43-C43)/6,2)</f>
         <v/>
       </c>
-      <c r="H43" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I43" s="6" t="n">
+      <c r="H43" s="11" t="inlineStr">
+        <is>
+          <t>RF-021</t>
+        </is>
+      </c>
+      <c r="I43" s="11" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="J43" s="11" t="n">
+        <v>36.08</v>
+      </c>
+      <c r="K43" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="J43" s="6" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="K43" s="6" t="n">
-        <v>35.17</v>
-      </c>
-      <c r="L43" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="L43" s="11" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>RNF-003</t>
+          <t>RNF-001</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Seguridad a nivel de fila (RLS)</t>
+          <t>Rendimiento del catálogo</t>
         </is>
       </c>
       <c r="C44" s="6" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F44" s="6">
         <f>ROUND((C44+4*D44+E44)/6,2)</f>
@@ -7601,17 +7803,17 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RF-007</t>
         </is>
       </c>
       <c r="I44" s="6" t="n">
-        <v>0</v>
+        <v>7.75</v>
       </c>
       <c r="J44" s="6" t="n">
-        <v>2.08</v>
+        <v>8.67</v>
       </c>
       <c r="K44" s="6" t="n">
-        <v>32.83</v>
+        <v>27.42</v>
       </c>
       <c r="L44" s="6" t="inlineStr">
         <is>
@@ -7622,22 +7824,22 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>RNF-004</t>
+          <t>RNF-002</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Confidencialidad de datos personales</t>
+          <t>Tokens de diseño</t>
         </is>
       </c>
       <c r="C45" s="6" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D45" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45" s="6">
         <f>ROUND((C45+4*D45+E45)/6,2)</f>
@@ -7649,17 +7851,17 @@
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>RNF-003</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I45" s="6" t="n">
-        <v>2.08</v>
+        <v>0</v>
       </c>
       <c r="J45" s="6" t="n">
-        <v>3.25</v>
+        <v>0.92</v>
       </c>
       <c r="K45" s="6" t="n">
-        <v>32.83</v>
+        <v>35.17</v>
       </c>
       <c r="L45" s="6" t="inlineStr">
         <is>
@@ -7670,22 +7872,22 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>RNF-005</t>
+          <t>RNF-003</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Sesión cifrada</t>
+          <t>Seguridad a nivel de fila (RLS)</t>
         </is>
       </c>
       <c r="C46" s="6" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F46" s="6">
         <f>ROUND((C46+4*D46+E46)/6,2)</f>
@@ -7704,10 +7906,10 @@
         <v>0</v>
       </c>
       <c r="J46" s="6" t="n">
-        <v>1.17</v>
+        <v>2.08</v>
       </c>
       <c r="K46" s="6" t="n">
-        <v>34.92</v>
+        <v>32.83</v>
       </c>
       <c r="L46" s="6" t="inlineStr">
         <is>
@@ -7718,19 +7920,19 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>RNF-006</t>
+          <t>RNF-004</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Mensajes en español</t>
+          <t>Confidencialidad de datos personales</t>
         </is>
       </c>
       <c r="C47" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E47" s="6" t="n">
         <v>2</v>
@@ -7745,17 +7947,17 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RNF-003</t>
         </is>
       </c>
       <c r="I47" s="6" t="n">
-        <v>0</v>
+        <v>2.08</v>
       </c>
       <c r="J47" s="6" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
       <c r="K47" s="6" t="n">
-        <v>34.58</v>
+        <v>32.83</v>
       </c>
       <c r="L47" s="6" t="inlineStr">
         <is>
@@ -7766,19 +7968,19 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>RNF-007</t>
+          <t>RNF-005</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Consistencia de la compra</t>
+          <t>Sesión cifrada</t>
         </is>
       </c>
       <c r="C48" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D48" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E48" s="6" t="n">
         <v>2</v>
@@ -7800,10 +8002,10 @@
         <v>0</v>
       </c>
       <c r="J48" s="6" t="n">
-        <v>1.83</v>
+        <v>1.17</v>
       </c>
       <c r="K48" s="6" t="n">
-        <v>34.25</v>
+        <v>34.92</v>
       </c>
       <c r="L48" s="6" t="inlineStr">
         <is>
@@ -7814,19 +8016,19 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>RNF-008</t>
+          <t>RNF-006</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Integración continua</t>
+          <t>Mensajes en español</t>
         </is>
       </c>
       <c r="C49" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E49" s="6" t="n">
         <v>2</v>
@@ -7848,10 +8050,10 @@
         <v>0</v>
       </c>
       <c r="J49" s="6" t="n">
-        <v>1.17</v>
+        <v>1.5</v>
       </c>
       <c r="K49" s="6" t="n">
-        <v>34.92</v>
+        <v>34.58</v>
       </c>
       <c r="L49" s="6" t="inlineStr">
         <is>
@@ -7862,19 +8064,19 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>RNF-009</t>
+          <t>RNF-007</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Accesibilidad</t>
+          <t>Consistencia de la compra</t>
         </is>
       </c>
       <c r="C50" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D50" s="6" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E50" s="6" t="n">
         <v>2</v>
@@ -7896,57 +8098,153 @@
         <v>0</v>
       </c>
       <c r="J50" s="6" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="K50" s="6" t="n">
+        <v>34.25</v>
+      </c>
+      <c r="L50" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>RNF-008</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Integración continua</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F51" s="6">
+        <f>ROUND((C51+4*D51+E51)/6,2)</f>
+        <v/>
+      </c>
+      <c r="G51" s="6">
+        <f>ROUND((E51-C51)/6,2)</f>
+        <v/>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="6" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="K51" s="6" t="n">
+        <v>34.92</v>
+      </c>
+      <c r="L51" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>RNF-009</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Accesibilidad</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="K50" s="6" t="n">
+      <c r="E52" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F52" s="6">
+        <f>ROUND((C52+4*D52+E52)/6,2)</f>
+        <v/>
+      </c>
+      <c r="G52" s="6">
+        <f>ROUND((E52-C52)/6,2)</f>
+        <v/>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K52" s="6" t="n">
         <v>34.58</v>
       </c>
-      <c r="L50" s="6" t="inlineStr">
+      <c r="L52" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="13" t="inlineStr">
-        <is>
-          <t>Total del proyecto (suma de TE)</t>
-        </is>
-      </c>
-      <c r="F52" s="13">
-        <f>SUM(F3:F50)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="13" t="inlineStr">
-        <is>
-          <t>Duración del camino crítico (días)</t>
-        </is>
-      </c>
-      <c r="F53" s="13" t="n">
-        <v>36.08</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>Camino crítico</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>RF-007 → RF-012 → RF-016 → RF-021 → RF-039</t>
-        </is>
+          <t>Total del proyecto (suma de TE)</t>
+        </is>
+      </c>
+      <c r="F54" s="13">
+        <f>SUM(F3:F52)</f>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="13" t="inlineStr">
         <is>
+          <t>Duración del camino crítico (días)</t>
+        </is>
+      </c>
+      <c r="F55" s="13" t="n">
+        <v>36.08</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="inlineStr">
+        <is>
+          <t>Camino crítico</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>RF-007 → RF-012 → RF-016 → RF-021 → RF-039</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
           <t>σ del camino crítico (días)</t>
         </is>
       </c>
-      <c r="F55" t="n">
+      <c r="F57" t="n">
         <v>2.43</v>
       </c>
     </row>
@@ -8015,7 +8313,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Etapa 1 - New You, secciones 7 y 8 (HU01–HU21). RF-011, RF-023, RF-025 a RF-028 y RF-035 todavía no tienen HU propia.</t>
+          <t>Etapa 1 - New You, secciones 7 y 8 (HU01–HU27). Todos los RF tienen al menos una HU.</t>
         </is>
       </c>
     </row>

</xml_diff>